<commit_message>
lab 8 updates and excel
</commit_message>
<xml_diff>
--- a/PRACTICE_8/a00_excel_crash_course.xlsx
+++ b/PRACTICE_8/a00_excel_crash_course.xlsx
@@ -1,16 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="28125"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
   <workbookPr date1904="1" showInkAnnotation="0" autoCompressPictures="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marce\OneDrive\Desktop\Masters_degree\AMD\ISEL_AMD_GRP06\TP8\ModuleOfPractice_08_LVQ\ModuleOfPractice_08_LVQ\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43D8F8A-AD0C-4222-BD45-5D2BAA06A0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30540" yWindow="1320" windowWidth="28280" windowHeight="16060" tabRatio="500"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="essential-techniques" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="140001" concurrentCalc="0"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -189,7 +206,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -331,70 +348,78 @@
     </xf>
   </cellXfs>
   <cellStyles count="61">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="44" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="46" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="48" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="50" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="52" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="54" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="56" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="58" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="60" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="43" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="45" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="47" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="49" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="51" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="53" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="55" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="57" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="59" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="43" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="45" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="47" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="49" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="51" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="53" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="55" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="57" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação" xfId="59" builtinId="8" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="44" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="46" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="48" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="50" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="52" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="54" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="56" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="58" builtinId="9" hidden="1"/>
+    <cellStyle name="Hiperligação Visitada" xfId="60" builtinId="9" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -717,37 +742,37 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R65"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.140625" customWidth="1"/>
-    <col min="7" max="10" width="6.140625" customWidth="1"/>
-    <col min="11" max="15" width="12.140625" customWidth="1"/>
-    <col min="16" max="16" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.1796875" customWidth="1"/>
+    <col min="7" max="10" width="6.1796875" customWidth="1"/>
+    <col min="11" max="15" width="12.1796875" customWidth="1"/>
+    <col min="16" max="16" width="18.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="6"/>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="6"/>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E4" s="6"/>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -756,11 +781,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E7" s="6"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
@@ -778,7 +803,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -814,7 +839,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -835,14 +860,32 @@
       <c r="J9">
         <v>4.5999999999999996</v>
       </c>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="K9" s="4">
+        <f>(G9-I9)^2</f>
+        <v>4.839999999999999</v>
+      </c>
+      <c r="L9" s="4">
+        <f>(H9-J9)^2</f>
+        <v>0.3599999999999996</v>
+      </c>
+      <c r="M9" s="4">
+        <f>K9+L9</f>
+        <v>5.1999999999999984</v>
+      </c>
+      <c r="N9" s="4">
+        <f>SQRT(M9)</f>
+        <v>2.2803508501982757</v>
+      </c>
+      <c r="O9" s="4">
+        <f>MIN(G9,H9)</f>
+        <v>4</v>
+      </c>
+      <c r="P9" s="4" t="str">
+        <f>IF(O9&gt;0,"&gt;0","&lt;=0")</f>
+        <v>&gt;0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E10" s="6"/>
       <c r="G10">
         <v>-7</v>
@@ -856,14 +899,32 @@
       <c r="J10">
         <v>-9.8000000000000007</v>
       </c>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="K10" s="4">
+        <f t="shared" ref="K10:K11" si="0">(G10-I10)^2</f>
+        <v>64</v>
+      </c>
+      <c r="L10" s="4">
+        <f t="shared" ref="L10:L11" si="1">(H10-J10)^2</f>
+        <v>96.04000000000002</v>
+      </c>
+      <c r="M10" s="4">
+        <f t="shared" ref="M10:M11" si="2">K10+L10</f>
+        <v>160.04000000000002</v>
+      </c>
+      <c r="N10" s="4">
+        <f>SQRT(M10)</f>
+        <v>12.650691680694775</v>
+      </c>
+      <c r="O10" s="4">
+        <f t="shared" ref="O10:O11" si="3">MIN(G10,H10)</f>
+        <v>-7</v>
+      </c>
+      <c r="P10" s="4" t="str">
+        <f t="shared" ref="P10:P11" si="4">IF(O10&gt;0,"&gt;0","&lt;=0")</f>
+        <v>&lt;=0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -880,14 +941,32 @@
       <c r="J11">
         <v>-3</v>
       </c>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-      <c r="P11" s="4"/>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="K11" s="4">
+        <f t="shared" si="0"/>
+        <v>2.4336000000000015</v>
+      </c>
+      <c r="L11" s="4">
+        <f t="shared" si="1"/>
+        <v>57.76</v>
+      </c>
+      <c r="M11" s="4">
+        <f t="shared" si="2"/>
+        <v>60.193599999999996</v>
+      </c>
+      <c r="N11" s="4">
+        <f t="shared" ref="N11" si="5">SQRT(M11)</f>
+        <v>7.7584534541363332</v>
+      </c>
+      <c r="O11" s="4">
+        <f t="shared" si="3"/>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="P11" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>&gt;0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1</v>
       </c>
@@ -899,33 +978,33 @@
       </c>
       <c r="E12" s="6"/>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13">
         <f>SUM(A12:C12)</f>
         <v>6</v>
       </c>
       <c r="E13" s="6"/>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E14" s="6"/>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="6"/>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16">
         <f>COUNT(A12:C12)</f>
         <v>3</v>
       </c>
       <c r="E16" s="6"/>
     </row>
-    <row r="17" spans="1:18">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="E17" s="6"/>
     </row>
-    <row r="18" spans="1:18">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -937,7 +1016,7 @@
       </c>
       <c r="E18" s="6"/>
     </row>
-    <row r="19" spans="1:18">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19">
         <f>2^2</f>
         <v>4</v>
@@ -952,10 +1031,10 @@
       </c>
       <c r="E19" s="6"/>
     </row>
-    <row r="20" spans="1:18">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="E20" s="6"/>
     </row>
-    <row r="21" spans="1:18">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -964,7 +1043,7 @@
       </c>
       <c r="E21" s="6"/>
     </row>
-    <row r="22" spans="1:18">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22">
         <f>EXP(2)</f>
         <v>7.3890560989306504</v>
@@ -975,29 +1054,29 @@
       </c>
       <c r="E22" s="6"/>
     </row>
-    <row r="23" spans="1:18">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="E23" s="6"/>
     </row>
-    <row r="24" spans="1:18">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>10</v>
       </c>
       <c r="E24" s="6"/>
     </row>
-    <row r="25" spans="1:18">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25">
         <f>PI()</f>
         <v>3.1415926535897931</v>
       </c>
       <c r="E25" s="6"/>
     </row>
-    <row r="26" spans="1:18">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="E26" s="6"/>
     </row>
-    <row r="27" spans="1:18">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="E27" s="6"/>
     </row>
-    <row r="28" spans="1:18">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
@@ -1039,7 +1118,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:18">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="E29" s="6"/>
       <c r="F29" s="7" t="s">
         <v>39</v>
@@ -1056,18 +1135,39 @@
       <c r="J29">
         <v>5.6</v>
       </c>
-      <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
-      <c r="M29" s="4"/>
-      <c r="N29" s="4"/>
+      <c r="K29" s="4">
+        <f>AVERAGE(G29:J29)</f>
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="L29" s="4">
+        <f>_xlfn.STDEV.P(G29:J29)</f>
+        <v>0.97339611669658643</v>
+      </c>
+      <c r="M29" s="4">
+        <f>_xlfn.MODE.SNGL(G29:J29)</f>
+        <v>5.6</v>
+      </c>
+      <c r="N29" s="4">
+        <f>MEDIAN(G29:J29)</f>
+        <v>4.8</v>
+      </c>
       <c r="O29" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="P29" s="4"/>
-      <c r="Q29" s="4"/>
-      <c r="R29" s="4"/>
-    </row>
-    <row r="30" spans="1:18">
+      <c r="P29" s="4">
+        <f>CORREL(G29:J29,G29:J29)</f>
+        <v>1</v>
+      </c>
+      <c r="Q29" s="4">
+        <f>CORREL(G30:J30,G29:J29)</f>
+        <v>-0.93297279273223688</v>
+      </c>
+      <c r="R29" s="4">
+        <f>CORREL(G31:J31,G29:J29)</f>
+        <v>-0.89163360435512151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -1087,18 +1187,39 @@
       <c r="J30">
         <v>-9.8000000000000007</v>
       </c>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
+      <c r="K30" s="4">
+        <f>AVERAGE(G30:J30)</f>
+        <v>-3.95</v>
+      </c>
+      <c r="L30" s="4">
+        <f>_xlfn.STDEV.P(G30:J30)</f>
+        <v>4.5724719791377622</v>
+      </c>
+      <c r="M30" s="4" t="e">
+        <f>_xlfn.MODE.SNGL(G30:J30)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N30" s="4">
+        <f t="shared" ref="N30:N31" si="6">MEDIAN(G30:J30)</f>
+        <v>-3.5</v>
+      </c>
       <c r="O30" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="P30" s="4"/>
-      <c r="Q30" s="4"/>
-      <c r="R30" s="4"/>
-    </row>
-    <row r="31" spans="1:18">
+      <c r="P30" s="4">
+        <f>CORREL(G29:J29,G30:J30)</f>
+        <v>-0.93297279273223688</v>
+      </c>
+      <c r="Q30" s="4">
+        <f>CORREL(G30:J30,G30:J30)</f>
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="R30" s="4">
+        <f>CORREL(G31:J31,G30:J30)</f>
+        <v>0.99466214345794257</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1</v>
       </c>
@@ -1124,34 +1245,55 @@
       <c r="J31">
         <v>5.3</v>
       </c>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
-      <c r="M31" s="4"/>
-      <c r="N31" s="4"/>
+      <c r="K31" s="4">
+        <f t="shared" ref="K31" si="7">AVERAGE(G31:J31)</f>
+        <v>11.009999999999998</v>
+      </c>
+      <c r="L31" s="4">
+        <f>_xlfn.STDEV.P(G31:J31)</f>
+        <v>4.3500919530511135</v>
+      </c>
+      <c r="M31" s="4" t="e">
+        <f>_xlfn.MODE.SNGL(G31:J31)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="N31" s="4">
+        <f t="shared" si="6"/>
+        <v>11.27</v>
+      </c>
       <c r="O31" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="P31" s="4"/>
-      <c r="Q31" s="4"/>
-      <c r="R31" s="4"/>
-    </row>
-    <row r="32" spans="1:18">
+      <c r="P31" s="4">
+        <f>CORREL(G29:J29,G31:J31)</f>
+        <v>-0.89163360435512151</v>
+      </c>
+      <c r="Q31" s="4">
+        <f>CORREL(G30:J30,G31:J31)</f>
+        <v>0.99466214345794257</v>
+      </c>
+      <c r="R31" s="4">
+        <f>CORREL(G31:J31,G31:J31)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32">
         <f>AVERAGE(A31:C31)</f>
         <v>2</v>
       </c>
       <c r="E32" s="6"/>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E33" s="6"/>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>13</v>
       </c>
       <c r="E34" s="6"/>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>1</v>
       </c>
@@ -1163,23 +1305,23 @@
       </c>
       <c r="E35" s="6"/>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <f>STDEV(A35:C35)</f>
         <v>1</v>
       </c>
       <c r="E36" s="6"/>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E37" s="6"/>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>45</v>
       </c>
       <c r="E38" s="6"/>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2</v>
       </c>
@@ -1191,23 +1333,23 @@
       </c>
       <c r="E39" s="6"/>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <f>MODE(A39:C39)</f>
         <v>2</v>
       </c>
       <c r="E40" s="6"/>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E41" s="6"/>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>46</v>
       </c>
       <c r="E42" s="6"/>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1</v>
       </c>
@@ -1222,29 +1364,29 @@
       </c>
       <c r="E43" s="6"/>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <f>MEDIAN(A43:D43)</f>
         <v>4.5</v>
       </c>
       <c r="E44" s="6"/>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E45" s="6"/>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>47</v>
       </c>
       <c r="E46" s="6"/>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>48</v>
       </c>
       <c r="E47" s="6"/>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2</v>
       </c>
@@ -1256,7 +1398,7 @@
       </c>
       <c r="E48" s="6"/>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>4</v>
       </c>
@@ -1268,83 +1410,83 @@
       </c>
       <c r="E49" s="6"/>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <f>PEARSON(A48:C48,A49:C49)</f>
         <v>1</v>
       </c>
       <c r="E50" s="6"/>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E51" s="6"/>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E52" s="6"/>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E53" s="6"/>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>15</v>
       </c>
       <c r="E54" s="6"/>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55">
         <f ca="1">RAND()</f>
-        <v>0.43525894607847582</v>
+        <v>0.10633897009222393</v>
       </c>
       <c r="E55" s="6"/>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E56" s="6"/>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>16</v>
       </c>
       <c r="E57" s="6"/>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58">
         <f ca="1">NORMINV(RAND(), 1, 1)</f>
-        <v>1.7783531104598058</v>
+        <v>-0.32224241687644506</v>
       </c>
       <c r="E58" s="6"/>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E59" s="6"/>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E60" s="6"/>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E61" s="6"/>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>18</v>
       </c>
       <c r="E62" s="6"/>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="str">
         <f>IF(1&gt;2,"YES","NO")</f>
         <v>NO</v>
       </c>
       <c r="E63" s="6"/>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E64" s="6"/>
     </row>
-    <row r="65" spans="5:5">
+    <row r="65" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E65" s="6"/>
     </row>
   </sheetData>

</xml_diff>